<commit_message>
fix strategic dot logic
</commit_message>
<xml_diff>
--- a/data/test_strategic.xlsx
+++ b/data/test_strategic.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>data</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -581,11 +581,7 @@
           <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
@@ -593,11 +589,7 @@
           <t>&lt; $100k</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="b">
         <v>1</v>
       </c>

</xml_diff>